<commit_message>
Update schema artifacts again
</commit_message>
<xml_diff>
--- a/project/excel/brc_schema.xlsx
+++ b/project/excel/brc_schema.xlsx
@@ -641,7 +641,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AQ1"/>
+  <dimension ref="A1:AR1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -742,120 +742,125 @@
       </c>
       <c r="T1" t="inlineStr">
         <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="U1" t="inlineStr">
+        <is>
           <t>description</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>abstract</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>relatedItem</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="X1" t="inlineStr">
         <is>
           <t>keywords</t>
         </is>
       </c>
-      <c r="X1" t="inlineStr">
+      <c r="Y1" t="inlineStr">
         <is>
           <t>datasetName</t>
         </is>
       </c>
-      <c r="Y1" t="inlineStr">
+      <c r="Z1" t="inlineStr">
         <is>
           <t>funding</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>dataset_url</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>issue</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>journal_license_url</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>journal_name</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>journal_open_access_flag</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>journal_type</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>journal_issn</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>volume</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>publication_date_text</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>publisher_information</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>country_publication_code</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>country_publication</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>conference_information</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>conference_type</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>conference_title</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>conference_location</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>conference_date</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>media</t>
         </is>

</xml_diff>

<commit_message>
Add dataset ontology annotations
</commit_message>
<xml_diff>
--- a/project/excel/brc_schema.xlsx
+++ b/project/excel/brc_schema.xlsx
@@ -10,14 +10,15 @@
     <sheet name="DatasetCollection" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Dataset" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Individual" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Contributor" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Funding" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="BRCOrganization" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Organism" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Plasmid" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="RelatedItem" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="MediaSet" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="MediaFile" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="OntologyAnnotation" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Contributor" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Funding" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="BRCOrganization" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Organism" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Plasmid" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="RelatedItem" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="MediaSet" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="MediaFile" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -449,6 +450,42 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:C1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>title</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>relatedItemType</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>relatedItemIdentifier</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <dataValidations count="1">
+    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"JournalArticle,Book,Dataset,Software,Thesis,Patent,Preprint,Presentation,Report,Webpage,WebApplication"</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:L1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
@@ -519,7 +556,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -641,7 +678,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AR1"/>
+  <dimension ref="A1:AS1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -767,100 +804,105 @@
       </c>
       <c r="Y1" t="inlineStr">
         <is>
+          <t>ontology_annotations</t>
+        </is>
+      </c>
+      <c r="Z1" t="inlineStr">
+        <is>
           <t>datasetName</t>
         </is>
       </c>
-      <c r="Z1" t="inlineStr">
+      <c r="AA1" t="inlineStr">
         <is>
           <t>funding</t>
         </is>
       </c>
-      <c r="AA1" t="inlineStr">
+      <c r="AB1" t="inlineStr">
         <is>
           <t>dataset_url</t>
         </is>
       </c>
-      <c r="AB1" t="inlineStr">
+      <c r="AC1" t="inlineStr">
         <is>
           <t>issue</t>
         </is>
       </c>
-      <c r="AC1" t="inlineStr">
+      <c r="AD1" t="inlineStr">
         <is>
           <t>journal_license_url</t>
         </is>
       </c>
-      <c r="AD1" t="inlineStr">
+      <c r="AE1" t="inlineStr">
         <is>
           <t>journal_name</t>
         </is>
       </c>
-      <c r="AE1" t="inlineStr">
+      <c r="AF1" t="inlineStr">
         <is>
           <t>journal_open_access_flag</t>
         </is>
       </c>
-      <c r="AF1" t="inlineStr">
+      <c r="AG1" t="inlineStr">
         <is>
           <t>journal_type</t>
         </is>
       </c>
-      <c r="AG1" t="inlineStr">
+      <c r="AH1" t="inlineStr">
         <is>
           <t>journal_issn</t>
         </is>
       </c>
-      <c r="AH1" t="inlineStr">
+      <c r="AI1" t="inlineStr">
         <is>
           <t>volume</t>
         </is>
       </c>
-      <c r="AI1" t="inlineStr">
+      <c r="AJ1" t="inlineStr">
         <is>
           <t>publication_date_text</t>
         </is>
       </c>
-      <c r="AJ1" t="inlineStr">
+      <c r="AK1" t="inlineStr">
         <is>
           <t>publisher_information</t>
         </is>
       </c>
-      <c r="AK1" t="inlineStr">
+      <c r="AL1" t="inlineStr">
         <is>
           <t>country_publication_code</t>
         </is>
       </c>
-      <c r="AL1" t="inlineStr">
+      <c r="AM1" t="inlineStr">
         <is>
           <t>country_publication</t>
         </is>
       </c>
-      <c r="AM1" t="inlineStr">
+      <c r="AN1" t="inlineStr">
         <is>
           <t>conference_information</t>
         </is>
       </c>
-      <c r="AN1" t="inlineStr">
+      <c r="AO1" t="inlineStr">
         <is>
           <t>conference_type</t>
         </is>
       </c>
-      <c r="AO1" t="inlineStr">
+      <c r="AP1" t="inlineStr">
         <is>
           <t>conference_title</t>
         </is>
       </c>
-      <c r="AP1" t="inlineStr">
+      <c r="AQ1" t="inlineStr">
         <is>
           <t>conference_location</t>
         </is>
       </c>
-      <c r="AQ1" t="inlineStr">
+      <c r="AR1" t="inlineStr">
         <is>
           <t>conference_date</t>
         </is>
       </c>
-      <c r="AR1" t="inlineStr">
+      <c r="AS1" t="inlineStr">
         <is>
           <t>media</t>
         </is>
@@ -935,38 +977,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F1"/>
+  <dimension ref="A1:C1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>contributorType</t>
+          <t>term_id</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>name</t>
+          <t>preferred_name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>email</t>
-        </is>
-      </c>
-      <c r="D1" t="inlineStr">
-        <is>
-          <t>primaryContact</t>
-        </is>
-      </c>
-      <c r="E1" t="inlineStr">
-        <is>
-          <t>affiliation</t>
-        </is>
-      </c>
-      <c r="F1" t="inlineStr">
-        <is>
-          <t>orcid</t>
+          <t>canonical_name</t>
         </is>
       </c>
     </row>
@@ -981,28 +1008,38 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:F1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>fundingOrganization</t>
+          <t>contributorType</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>awardNumber</t>
+          <t>name</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>awardTitle</t>
+          <t>email</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>awardURI</t>
+          <t>primaryContact</t>
+        </is>
+      </c>
+      <c r="E1" t="inlineStr">
+        <is>
+          <t>affiliation</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>orcid</t>
         </is>
       </c>
     </row>
@@ -1023,22 +1060,22 @@
     <row r="1">
       <c r="A1" t="inlineStr">
         <is>
-          <t>organizationName</t>
+          <t>fundingOrganization</t>
         </is>
       </c>
       <c r="B1" t="inlineStr">
         <is>
-          <t>parentOrganization</t>
+          <t>awardNumber</t>
         </is>
       </c>
       <c r="C1" t="inlineStr">
         <is>
-          <t>wikidata_id</t>
+          <t>awardTitle</t>
         </is>
       </c>
       <c r="D1" t="inlineStr">
         <is>
-          <t>ror_id</t>
+          <t>awardURI</t>
         </is>
       </c>
     </row>
@@ -1048,6 +1085,42 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D1"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>organizationName</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>parentOrganization</t>
+        </is>
+      </c>
+      <c r="C1" t="inlineStr">
+        <is>
+          <t>wikidata_id</t>
+        </is>
+      </c>
+      <c r="D1" t="inlineStr">
+        <is>
+          <t>ror_id</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1078,7 +1151,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1132,40 +1205,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:C1"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
-        <is>
-          <t>title</t>
-        </is>
-      </c>
-      <c r="B1" t="inlineStr">
-        <is>
-          <t>relatedItemType</t>
-        </is>
-      </c>
-      <c r="C1" t="inlineStr">
-        <is>
-          <t>relatedItemIdentifier</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <dataValidations count="1">
-    <dataValidation sqref="B2:B1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"JournalArticle,Book,Dataset,Software,Thesis,Patent,Preprint,Presentation,Report,Webpage,WebApplication"</formula1>
-    </dataValidation>
-  </dataValidations>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Deprecate category slot, require topic, expand DatasetTopicEnum
Addresses part of #147.

- Mark the `category` slot as deprecated in favor of `topic`; it is
  retained only for backward compatibility with existing data feeds.
- Make `topic` required. This is a breaking change, so bump the schema
  version 0.1.15 -> 0.2.0.
- Expand DatasetTopicEnum with four OSTI-Subject-derived values that are
  semantically distinct from the existing eight: Environmental Science &
  Sustainability, Chemistry, Materials Science & Bioproducts, and
  Computational Biology & Modeling.
- Record the corresponding OSTI subject category code on each topic via
  an annotation, sourced from the bioenergy.org #236 investigation.
- Add a topic to the JBEI plasmid example so it remains valid under the
  new required constraint.
- Regenerate derived project artifacts and the Python datamodel.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/project/excel/brc_schema.xlsx
+++ b/project/excel/brc_schema.xlsx
@@ -909,7 +909,7 @@
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="4">
     <dataValidation sqref="H2:H1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"CABBI,CBI,GLBRC,JBEI"</formula1>
     </dataValidation>
@@ -918,9 +918,6 @@
     </dataValidation>
     <dataValidation sqref="Q2:Q1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"AS,GD,IM,ND,IP,FP,SM,MM,I"</formula1>
-    </dataValidation>
-    <dataValidation sqref="R2:R1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Genetic Engineering,Plant Biology,Microbiology,Analytics &amp; Methods,Enzymes &amp; Proteins,Biomass &amp; Feedstock,Bioenergy Production,Process Engineering"</formula1>
     </dataValidation>
     <dataValidation sqref="S2:S1048576" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Feedstock Development,Deconstruction and Separation,Conversion,Sustainability"</formula1>

</xml_diff>